<commit_message>
chore(daily): 自动更新 data.js + stock_data.xlsx (北京时间 2026-09-02 03:10)
</commit_message>
<xml_diff>
--- a/stock_data.xlsx
+++ b/stock_data.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L484"/>
+  <dimension ref="A1:L485"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20757,6 +20757,48 @@
       </c>
       <c r="L484" t="n">
         <v>-0.02641589180050719</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>600276.SH</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C485" t="n">
+        <v>46.05</v>
+      </c>
+      <c r="D485" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="E485" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="F485" t="n">
+        <v>46.23</v>
+      </c>
+      <c r="G485" t="n">
+        <v>46.07</v>
+      </c>
+      <c r="H485" t="n">
+        <v>0.1599999999999966</v>
+      </c>
+      <c r="I485" t="n">
+        <v>0.3472975906229576</v>
+      </c>
+      <c r="J485" t="n">
+        <v>46519265</v>
+      </c>
+      <c r="K485" t="n">
+        <v>2146398900</v>
+      </c>
+      <c r="L485" t="n">
+        <v>0.003472975906229525</v>
       </c>
     </row>
   </sheetData>
@@ -20770,7 +20812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L484"/>
+  <dimension ref="A1:L485"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41111,6 +41153,48 @@
       </c>
       <c r="L484" t="n">
         <v>-0.02641589180050719</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>600276.SH</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C485" t="n">
+        <v>46.05</v>
+      </c>
+      <c r="D485" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="E485" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="F485" t="n">
+        <v>46.23</v>
+      </c>
+      <c r="G485" t="n">
+        <v>46.07</v>
+      </c>
+      <c r="H485" t="n">
+        <v>0.1599999999999966</v>
+      </c>
+      <c r="I485" t="n">
+        <v>0.3472975906229576</v>
+      </c>
+      <c r="J485" t="n">
+        <v>46519265</v>
+      </c>
+      <c r="K485" t="n">
+        <v>2146398900</v>
+      </c>
+      <c r="L485" t="n">
+        <v>0.003472975906229525</v>
       </c>
     </row>
   </sheetData>
@@ -41124,7 +41208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L484"/>
+  <dimension ref="A1:L485"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61465,6 +61549,48 @@
       </c>
       <c r="L484" t="n">
         <v>0.006008583690987113</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>000001.SZ</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C485" t="n">
+        <v>11.68</v>
+      </c>
+      <c r="D485" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="E485" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="F485" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="G485" t="n">
+        <v>11.72</v>
+      </c>
+      <c r="H485" t="n">
+        <v>0.1999999999999993</v>
+      </c>
+      <c r="I485" t="n">
+        <v>1.706484641638219</v>
+      </c>
+      <c r="J485" t="n">
+        <v>153157153</v>
+      </c>
+      <c r="K485" t="n">
+        <v>1807254400</v>
+      </c>
+      <c r="L485" t="n">
+        <v>0.01706484641638228</v>
       </c>
     </row>
   </sheetData>
@@ -61478,7 +61604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L484"/>
+  <dimension ref="A1:L485"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81821,6 +81947,48 @@
         <v>0.006008583690987113</v>
       </c>
     </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>000001.SZ</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C485" t="n">
+        <v>11.68</v>
+      </c>
+      <c r="D485" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="E485" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="F485" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="G485" t="n">
+        <v>11.72</v>
+      </c>
+      <c r="H485" t="n">
+        <v>0.1999999999999993</v>
+      </c>
+      <c r="I485" t="n">
+        <v>1.706484641638219</v>
+      </c>
+      <c r="J485" t="n">
+        <v>153157153</v>
+      </c>
+      <c r="K485" t="n">
+        <v>1807254400</v>
+      </c>
+      <c r="L485" t="n">
+        <v>0.01706484641638228</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(daily): 自动更新 data.js + stock_data.xlsx (北京时间 2026-09-03 03:11)
</commit_message>
<xml_diff>
--- a/stock_data.xlsx
+++ b/stock_data.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L485"/>
+  <dimension ref="A1:L486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20799,6 +20799,48 @@
       </c>
       <c r="L485" t="n">
         <v>0.003472975906229525</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>600276.SH</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>46.23</v>
+      </c>
+      <c r="D486" t="n">
+        <v>46.32</v>
+      </c>
+      <c r="E486" t="n">
+        <v>45.49</v>
+      </c>
+      <c r="F486" t="n">
+        <v>45.57</v>
+      </c>
+      <c r="G486" t="n">
+        <v>46.23</v>
+      </c>
+      <c r="H486" t="n">
+        <v>-0.6599999999999966</v>
+      </c>
+      <c r="I486" t="n">
+        <v>-1.427644386761836</v>
+      </c>
+      <c r="J486" t="n">
+        <v>54670678</v>
+      </c>
+      <c r="K486" t="n">
+        <v>2509384100</v>
+      </c>
+      <c r="L486" t="n">
+        <v>-0.01427644386761839</v>
       </c>
     </row>
   </sheetData>
@@ -20812,7 +20854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L485"/>
+  <dimension ref="A1:L486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41195,6 +41237,48 @@
       </c>
       <c r="L485" t="n">
         <v>0.003472975906229525</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>600276.SH</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>46.23</v>
+      </c>
+      <c r="D486" t="n">
+        <v>46.32</v>
+      </c>
+      <c r="E486" t="n">
+        <v>45.49</v>
+      </c>
+      <c r="F486" t="n">
+        <v>45.57</v>
+      </c>
+      <c r="G486" t="n">
+        <v>46.23</v>
+      </c>
+      <c r="H486" t="n">
+        <v>-0.6599999999999966</v>
+      </c>
+      <c r="I486" t="n">
+        <v>-1.427644386761836</v>
+      </c>
+      <c r="J486" t="n">
+        <v>54670678</v>
+      </c>
+      <c r="K486" t="n">
+        <v>2509384100</v>
+      </c>
+      <c r="L486" t="n">
+        <v>-0.01427644386761839</v>
       </c>
     </row>
   </sheetData>
@@ -41208,7 +41292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L485"/>
+  <dimension ref="A1:L486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61591,6 +61675,48 @@
       </c>
       <c r="L485" t="n">
         <v>0.01706484641638228</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>000001.SZ</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="D486" t="n">
+        <v>11.99</v>
+      </c>
+      <c r="E486" t="n">
+        <v>11.85</v>
+      </c>
+      <c r="F486" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="G486" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H486" t="n">
+        <v>-0.009999999999999787</v>
+      </c>
+      <c r="I486" t="n">
+        <v>-0.08389261744966264</v>
+      </c>
+      <c r="J486" t="n">
+        <v>89237247</v>
+      </c>
+      <c r="K486" t="n">
+        <v>1063261800</v>
+      </c>
+      <c r="L486" t="n">
+        <v>-0.000838926174496657</v>
       </c>
     </row>
   </sheetData>
@@ -61604,7 +61730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L485"/>
+  <dimension ref="A1:L486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81989,6 +82115,48 @@
         <v>0.01706484641638228</v>
       </c>
     </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>000001.SZ</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="D486" t="n">
+        <v>11.99</v>
+      </c>
+      <c r="E486" t="n">
+        <v>11.85</v>
+      </c>
+      <c r="F486" t="n">
+        <v>11.91</v>
+      </c>
+      <c r="G486" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H486" t="n">
+        <v>-0.009999999999999787</v>
+      </c>
+      <c r="I486" t="n">
+        <v>-0.08389261744966264</v>
+      </c>
+      <c r="J486" t="n">
+        <v>89237247</v>
+      </c>
+      <c r="K486" t="n">
+        <v>1063261800</v>
+      </c>
+      <c r="L486" t="n">
+        <v>-0.000838926174496657</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>